<commit_message>
feat: reconhecer empresas por origem na importacao
</commit_message>
<xml_diff>
--- a/public/modelo-empresas.xlsx
+++ b/public/modelo-empresas.xlsx
@@ -44,9 +44,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <cols>
-    <col min="1" max="8" width="22" style="1" customWidth="1"/>
+    <col min="1" max="9" width="22" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -88,6 +88,11 @@
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>cnae_principal</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>google_place_id</t>
         </is>
       </c>
     </row>
@@ -132,6 +137,11 @@
           <t>4742300</t>
         </is>
       </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>ChIJ-ficticio-aurora</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
feat: listas de prospecção com CNPJ opcional (#50)
* docs: registrar plano aprovado de prospeccao por grupos

* feat: permitir identificacao cadastral parcial de empresas

* feat: reconhecer empresas por origem na importacao

* fix: preservar selecao conferida na importacao

* fix: compactar estado enviado na confirmacao

* feat: registrar e corrigir o contexto das listas importadas

* feat: restringir consulta e reserva ao grupo selecionado

* fix: preservar filtros ao abrir escolha de lista

* fix: alinhar props de pagina whatsapp ao contrato next

* feat: apresentar listas de prospeccao com origem e disponibilidade

* feat: preparar coleta da Mooca para importacao rastreavel

* docs: registrar execucao e evidencias da prospeccao

* fix(empresas): recusar aliases da mesma empresa na conferência

* docs: registrar verificacao final da prospeccao

* docs: atualizar referencias dos commits privados
</commit_message>
<xml_diff>
--- a/public/modelo-empresas.xlsx
+++ b/public/modelo-empresas.xlsx
@@ -44,9 +44,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <cols>
-    <col min="1" max="8" width="22" style="1" customWidth="1"/>
+    <col min="1" max="9" width="22" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -88,6 +88,11 @@
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>cnae_principal</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>google_place_id</t>
         </is>
       </c>
     </row>
@@ -132,6 +137,11 @@
           <t>4742300</t>
         </is>
       </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>ChIJ-ficticio-aurora</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>